<commit_message>
Add slider taste questions to onboarding behind a flag
Six taste sliders with 30 food pictures, a semi-circle swap animation, snap on release, Skip for now on every question, Skip the rest from the fourth, typed-in question text with a tick per letter, and one 22-screen progress bar. Answered tastes are passed to the dietary step so skipped ones are recorded as not set. Re-scored teh tarik, kopi and mee siam sweetness in the answer key.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013gNoSSagZkZJiocrmGMfpP
</commit_message>
<xml_diff>
--- a/data/taste-answer-key.xlsx
+++ b/data/taste-answer-key.xlsx
@@ -1298,7 +1298,7 @@
         </is>
       </c>
       <c r="C21" s="65" t="n">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="D21" s="65" t="n">
         <v>5</v>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="C33" s="65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D33" s="65" t="n">
         <v>0</v>
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="C34" s="66" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="D34" s="66" t="n">
         <v>0</v>

</xml_diff>